<commit_message>
suppression pages et artefacts (#116)
* suppression pages et artefacts

* Modifications editoriales 2eea62a3382fbb9647a2066d3901ae8b97e6d43d
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-inpatient-medication-dispense.xlsx
+++ b/main/ig/StructureDefinition-fr-inpatient-medication-dispense.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-19T09:10:48+00:00</t>
+    <t>2026-05-27T13:03:41+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -824,7 +824,7 @@
     <t>MedicationDispense.authorizingPrescription</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/medication/StructureDefinition/fr-inpatient-medicationrequest)
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/eprescription/StructureDefinition/fr-inpatient-medicationrequest)
 </t>
   </si>
   <si>
@@ -1477,7 +1477,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="74.48828125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="89.47265625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>